<commit_message>
W01 D4 workbook: the Share tab reads both directions against a reading agreed before the test, with no 0.05 line; the Count tab counts customers and says worth testing on its count; recalc manifest re-proved
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W01/D4/demos/C2_W01_D04_decision_tool_STUDENT.xlsx
+++ b/content/W01/D4/demos/C2_W01_D04_decision_tool_STUDENT.xlsx
@@ -525,7 +525,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Share: what a p-value says. Size: whether a real gap is worth acting on. Count: whether a rate is a finding or a lead. Mix: whether the campaign worked once the segments are split.</t>
+          <t>Share: what a share says, in both directions. Size: whether a real gap is worth acting on. Count: whether a rate is a lead or worth testing, counted in customers. Mix: whether the campaign worked once the segments are split.</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Shuffle the segment labels many times and count how often chance alone makes a gap this large. The numbers are invented, change them.</t>
+          <t>Flip each member's pair many times (or shuffle the labels, for different customers) and count how often chance alone makes a gap this large, one way and either way. The numbers are invented, change them.</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shuffles run</t>
+          <t>Flips run</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -595,83 +595,150 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shuffles at least as large as the real gap</t>
+          <t>Flips with a fall at least as large as the real one</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
         <v>210</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Flips with a move that large in either direction</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>400</v>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>The share (the p-value)</t>
-        </is>
-      </c>
-      <c r="B8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>The direction the team decided before the test</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>not decided before the test</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Agreed before the test: a share below this reads as rare</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Agreed before the test: a share above this reads as the usual wobble</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>The share, falls only</t>
+        </is>
+      </c>
+      <c r="B12">
         <f>B6/1000</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>The share, either way</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>B7/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>The share the verdict reads</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(B8="falls only",B12,B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
       </c>
-      <c r="B9" s="2">
-        <f>IF(AND(B8&gt;=0,B8&lt;=1,ABS(B8-B6/B5)&lt;0.0000001),"The share is the count at least as large, over the shuffles run.","The share is outside 0 to 1 or differs from the count over the shuffles: it divides by the wrong cell. Fix it first.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="B15" s="2">
+        <f>IF(AND(B12&gt;=0,B12&lt;=1,ABS(B12-B6/B5)&lt;0.0000001),"The share is the count at least as large, over the flips run.","The share is outside 0 to 1 or differs from the count over the flips: it divides by the wrong cell. Fix it first.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>The sentence you would write</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>a X percent chance we are wrong</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Is it defensible?</t>
         </is>
       </c>
-      <c r="B12" s="2">
-        <f>IF(B11="X of every 100 chance-only worlds","Defensible: the share counts chance-only worlds, which is all a p-value measures.","Indefensible: a p-value is a share of chance-only worlds, never the chance the finding is wrong. Choose the chance-only worlds sentence.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="B18" s="2">
+        <f>IF(B17="X of every 100 chance-only worlds","Defensible: the share counts chance-only worlds, which is all a p-value measures.","Indefensible: a p-value is a share of chance-only worlds, and it cannot be the chance the finding is wrong. Choose the chance-only worlds sentence.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B14" s="8">
-        <f>IF(ABS(B8-B6/B5)&gt;=0.0000001,"Fix the share formula before reading the verdict.",IF(B8&lt;0.05,"Chance makes a gap this large in about "&amp;TEXT(B8*100,"0.0")&amp;" of every 100 shuffles, so treat it as real and size it next.","Chance makes a gap this large in about "&amp;TEXT(B8*100,"0.0")&amp;" of every 100 shuffles: inside the usual wobble, so not yet."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B20" s="8">
+        <f>IF(ABS(B12-B6/B5)&gt;=0.0000001,"Fix the share formula before reading the verdict.",IF(B8="falls only","Counting falls only, as decided before the test, chance makes a fall this large in about "&amp;TEXT(B12*100,"0.0")&amp;" of every 100 flips, and a move that large either way in about "&amp;TEXT(B13*100,"0.0")&amp;". ",IF(B8="either way","Counting either way, as decided before the test, chance makes a move this large in about "&amp;TEXT(B13*100,"0.0")&amp;" of every 100 flips, and a fall this large in about "&amp;TEXT(B12*100,"0.0")&amp;". ","No direction was decided before the test, so both go in the note: a fall this large turns up in about "&amp;TEXT(B12*100,"0.0")&amp;" of every 100 flips, and a move that large either way in about "&amp;TEXT(B13*100,"0.0")&amp;". "))&amp;IF(B14&lt;B9,"By the reading agreed before the test, that is rare as pure wobble, so size it next.",IF(B14&lt;=B10,"By the reading agreed before the test, that is borderline: size it, and watch it before acting on it alone.","By the reading agreed before the test, that is inside the usual wobble, so not yet.")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
       </c>
-      <c r="B15">
-        <f>IF(ABS(B8-B6/B5)&lt;0.0000001,1,0)</f>
+      <c r="B21">
+        <f>IF(ABS(B12-B6/B5)&lt;0.0000001,1,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"falls only,either way,not decided before the test"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"a X percent chance we are wrong,X of every 100 chance-only worlds,X percent certain"</formula1>
     </dataValidation>
   </dataValidations>
@@ -858,7 +925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -870,14 +937,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Is the rate a finding or a lead?</t>
+          <t>Is the rate a lead, or worth testing?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>A rate that jumps by 40 percent can stand on a handful of orders. Count what it stands on first. The numbers are invented, change them.</t>
+          <t>A rate that jumps by 40 percent can stand on a handful of orders from a handful of customers. Count both first; the rule of thumb counts customers, since more orders from the same few customers add no new evidence. The numbers are invented, change them.</t>
         </is>
       </c>
     </row>
@@ -913,80 +980,90 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Customers who placed those orders</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Rate change, percent</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B9">
         <f>100*(B6-B5)/B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Orders the rate stands on</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>B5+B6</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>One-order swing, points</t>
+          <t>Orders the rate stands on</t>
         </is>
       </c>
       <c r="B10">
-        <f>100/B9</f>
+        <f>B5+B6</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>One-order swing, points</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>100/B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>The call</t>
         </is>
       </c>
-      <c r="B11">
-        <f>IF(B8&lt;30,"lead","finding")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B12">
+        <f>IF(B9&lt;30,"lead","worth testing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
       </c>
-      <c r="B12" s="2">
-        <f>IF(B11=IF(B9&lt;30,"lead","finding"),"The call reads the count of orders against thirty.","The call and the count disagree: the threshold test reads the rate where it should read the count. Fix it first.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="B13" s="2">
+        <f>IF(B12=IF(B7&lt;30,"lead","worth testing"),"The call reads the customers behind the rate against thirty.","The call and the count disagree: the threshold test reads the rate where it should read the customers. Fix it first.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B14" s="8">
-        <f>IF(B11&lt;&gt;IF(B9&lt;30,"lead","finding"),"Fix the threshold test before calling the rate.",IF(B9&lt;30,"A rise of "&amp;TEXT(B8,"0.0")&amp;" percent on "&amp;B9&amp;" orders is a lead: watch it until it carries thirty or more. One order moves it by about "&amp;TEXT(B10,"0.0")&amp;" points.","A rise of "&amp;TEXT(B8,"0.0")&amp;" percent on "&amp;B9&amp;" orders is a finding worth testing."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B15" s="8">
+        <f>IF(B12&lt;&gt;IF(B7&lt;30,"lead","worth testing"),"Fix the threshold test before calling the rate.",IF(B7&lt;30,"A rise of "&amp;TEXT(B9,"0.0")&amp;" percent on "&amp;B10&amp;" orders from "&amp;B7&amp;" customers is a lead: watch it until more customers buy, thirty or more, since more orders from the same few customers add no new evidence. One order moves it by about "&amp;TEXT(B11,"0.0")&amp;" points.","A rise of "&amp;TEXT(B9,"0.0")&amp;" percent on "&amp;B10&amp;" orders from "&amp;B7&amp;" customers is worth testing on its count."))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
       </c>
-      <c r="B15">
-        <f>IF(B11=IF(B9&lt;30,"lead","finding"),1,0)</f>
+      <c r="B16">
+        <f>IF(B12=IF(B7&lt;30,"lead","worth testing"),1,0)</f>
         <v/>
       </c>
     </row>
@@ -1229,7 +1306,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>Share!B15+Size!B18+Count!B15+Mix!B19</f>
+        <f>Share!B21+Size!B18+Count!B16+Mix!B19</f>
         <v/>
       </c>
     </row>
@@ -1251,7 +1328,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>IF(B4=4,"Share: "&amp;Share!B14&amp;CHAR(10)&amp;"Size: "&amp;Size!B17&amp;CHAR(10)&amp;"Count: "&amp;Count!B14&amp;CHAR(10)&amp;"Mix: "&amp;Mix!B18,"The note assembles once every tab passes its check.")</f>
+        <f>IF(B4=4,"Share: "&amp;Share!B20&amp;CHAR(10)&amp;"Size: "&amp;Size!B17&amp;CHAR(10)&amp;"Count: "&amp;Count!B15&amp;CHAR(10)&amp;"Mix: "&amp;Mix!B18,"The note assembles once every tab passes its check.")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
W01 D4 reading family mid-raise, saved as the agent stands: notes, cheat sheet, board work, pre-read, extras, companion page and workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FuBiPzJ5MbkU3CtQUt4t8P
</commit_message>
<xml_diff>
--- a/content/W01/D4/demos/C2_W01_D04_decision_tool_STUDENT.xlsx
+++ b/content/W01/D4/demos/C2_W01_D04_decision_tool_STUDENT.xlsx
@@ -36,16 +36,16 @@
       <sz val="16"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001A0F5C"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="006B6690"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001A0F5C"/>
     </font>
     <font>
       <b val="1"/>
@@ -109,9 +109,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -490,21 +490,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Before the growth review: the decision tool</t>
+          <t>Which four decisions stand between Meera's three questions and her note?</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kalpa Retail, Week 1, Thursday. Meera asks three things before Monday's growth review: is the Retail-Plus drop real or the usual wobble, should budget follow a segment that is up 40 percent, and did the monsoon discount work. Four decisions answer her, one tab each, and an Export tab assembles the note.</t>
+          <t>Kalpa Retail, Week 1, Thursday. Meera Raghavan, the CEO, asks three things before Monday's growth review: is the fall in Retail-Plus, Kalpa's paid membership tier, real or the usual wobble; should budget follow a segment that is up 40 percent; and did the monsoon discount work? Four decisions answer her, one tab each, and an Export tab assembles the note.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Yellow cells are inputs; every other number and sentence is a live formula. Every number here is invented, so change it and watch the verdict move.</t>
+          <t>Yellow cells are inputs, and every other number and sentence is a live formula. Every number here is invented, so change it and watch the verdict move.</t>
         </is>
       </c>
     </row>
@@ -522,15 +522,50 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Share: what a share says, in both directions. Size: whether a real gap is worth acting on. Count: whether a rate is a lead or worth testing, counted in customers. Mix: whether the campaign worked once the segments are split.</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Which question does each tab answer?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Share: how often does chance alone make a fall this large, and which sentence says so honestly?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Size: is a fall that beats chance worth more than the fix costs?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Count: is a rate that rose a lead, or worth testing, once you count its customers?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Mix: did the campaign raise spend inside each group, or only in the blend?</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Export: is every tab fixed, and what does the note to Meera say?</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>The note to Meera runs claim, evidence, caveat, action, and each verdict is written to sit inside it.</t>
         </is>
@@ -559,24 +594,24 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What does the share say?</t>
+          <t>How often does chance alone make a fall this large, and which sentence says so honestly?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Flip each member's pair many times (or shuffle the labels, for different customers) and count how often chance alone makes a gap this large, one way and either way. The numbers are invented, change them.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Flip each member's pair many times (or shuffle the labels, for different customers) and count how often chance alone makes a gap this large, one way and either way. The numbers are invented; change them.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -588,7 +623,7 @@
           <t>Flips run</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -598,7 +633,7 @@
           <t>Flips with a fall at least as large as the real one</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>210</v>
       </c>
     </row>
@@ -608,7 +643,7 @@
           <t>Flips with a move that large in either direction</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>400</v>
       </c>
     </row>
@@ -618,7 +653,7 @@
           <t>The direction the team decided before the test</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>not decided before the test</t>
         </is>
@@ -630,7 +665,7 @@
           <t>Agreed before the test: a share below this reads as rare</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -640,12 +675,12 @@
           <t>Agreed before the test: a share above this reads as the usual wobble</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>The share, falls only</t>
         </is>
@@ -656,7 +691,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>The share, either way</t>
         </is>
@@ -678,7 +713,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
@@ -689,12 +724,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>The sentence you would write</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>a X percent chance we are wrong</t>
         </is>
@@ -723,7 +758,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
@@ -764,24 +799,24 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Is it worth acting on?</t>
+          <t>Is a fall that beats chance worth more than the fix costs?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Real and worth acting on are two separate calls. Size the fall in rupees against the cost of the fix. The numbers are invented, change them.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Real and worth acting on are two separate calls. Size the fall in rupees against the cost of the fix. The numbers are invented; change them.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -793,7 +828,7 @@
           <t>Gap per member in the quarter (Rs)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>160</v>
       </c>
     </row>
@@ -803,7 +838,7 @@
           <t>Members in the segment</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>7000</v>
       </c>
     </row>
@@ -813,7 +848,7 @@
           <t>Company revenue in the quarter (Rs)</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>95000000</v>
       </c>
     </row>
@@ -823,7 +858,7 @@
           <t>Cost of acting per quarter (Rs)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>250000</v>
       </c>
     </row>
@@ -833,12 +868,12 @@
           <t>Share of the fall the fix wins back, percent</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Segment fall in the quarter (Rs)</t>
         </is>
@@ -882,7 +917,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
@@ -904,7 +939,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
@@ -937,24 +972,24 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Is the rate a lead, or worth testing?</t>
+          <t>Is a rate that rose a lead, or worth testing, once you count its customers?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>A rate that jumps by 40 percent can stand on a handful of orders from a handful of customers. Count both first; the rule of thumb counts customers, since more orders from the same few customers add no new evidence. The numbers are invented, change them.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>A rate that jumps by 40 percent can stand on a handful of orders from a handful of customers. Count both first; the rule of thumb counts customers, since more orders from the same few customers add no new evidence. The numbers are invented; change them.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -966,7 +1001,7 @@
           <t>Orders in the earlier quarter</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -976,7 +1011,7 @@
           <t>Orders in the later quarter</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -986,12 +1021,12 @@
           <t>Customers who placed those orders</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Rate change, percent</t>
         </is>
@@ -1035,7 +1070,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
@@ -1057,7 +1092,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
@@ -1090,34 +1125,34 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Did the campaign work?</t>
+          <t>Did the campaign raise spend inside each group, or only in the blend?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Split the aggregate by segment before crediting a campaign. Two invented groups, spend per customer in the quarter; change them.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>The blend is one average over both groups mixed together, so a campaign that reached more big spenders can raise it while every group spends less. Split by group before crediting the campaign. The spend per customer in the quarter is invented; change it.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Not exposed (Rs)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Exposed (Rs)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Change (Rs)</t>
         </is>
@@ -1129,10 +1164,10 @@
           <t>big spenders</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>5000</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <v>4700</v>
       </c>
       <c r="D5">
@@ -1146,10 +1181,10 @@
           <t>small spenders</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>900</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="n">
         <v>850</v>
       </c>
       <c r="D6">
@@ -1163,7 +1198,7 @@
           <t>Big spenders in the not-exposed group, percent</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1173,12 +1208,12 @@
           <t>Big spenders in the exposed group, percent</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Blended, not exposed (Rs)</t>
         </is>
@@ -1189,7 +1224,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Blended, exposed (Rs)</t>
         </is>
@@ -1233,7 +1268,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
@@ -1255,7 +1290,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
@@ -1288,19 +1323,19 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The note, assembled</t>
+          <t>Is every tab fixed, and what does the note to Meera say?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Released only when every tab's check passes. Paste the lines into the note to Meera as claim, evidence, caveat and action.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>The note is released only when every tab's check passes. Paste its lines into the note to Meera as claim, evidence, caveat and action.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tabs fixed</t>
         </is>
@@ -1322,7 +1357,7 @@
       </c>
     </row>
     <row r="7" ht="120" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Paste-ready note</t>
         </is>

</xml_diff>

<commit_message>
W01 D4 reading family after the review: the notes ask the new question 6 wordings and answer them, name the drawing, drop a saying, a bold label and two remarks about the document, and give the protected figures exactly; the cheat sheet's panels explain route, lead, blend and the audit and still print the vocabulary strip; the pre-read, board work, companion page, extras and workbook lose their staged lines and explain their terms; the companion's experiment A flips the same members
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FuBiPzJ5MbkU3CtQUt4t8P
</commit_message>
<xml_diff>
--- a/content/W01/D4/demos/C2_W01_D04_decision_tool_STUDENT.xlsx
+++ b/content/W01/D4/demos/C2_W01_D04_decision_tool_STUDENT.xlsx
@@ -546,7 +546,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Count: is a rate that rose a lead, or worth testing, once you count its customers?</t>
+          <t>Count: is a rate that rose worth testing, or only worth watching, once you count its customers?</t>
         </is>
       </c>
     </row>
@@ -972,14 +972,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Is a rate that rose a lead, or worth testing, once you count its customers?</t>
+          <t>Is a rate that rose worth testing, or only worth watching, once you count its customers?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>A rate that jumps by 40 percent can stand on a handful of orders from a handful of customers. Count both first; the rule of thumb counts customers, since more orders from the same few customers add no new evidence. The numbers are invented; change them.</t>
+          <t>A rate that jumps by 40 percent can stand on a handful of orders from a handful of customers. Count both first; the rule of thumb counts customers, since more orders from the same few customers add no new evidence, and a rate on fewer than thirty customers is a lead, one to watch until more customers buy. The numbers are invented; change them.</t>
         </is>
       </c>
     </row>

</xml_diff>